<commit_message>
Enriquecer reglas de hospitales: +53 nuevas variantes de direcciones y completar Hospital_final en reglas existentes
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reglas_hospitales.xlsx
+++ b/Reglas_hospitales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CANDIDATOS_HOSPITALES" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CANDIDATOS_FEDERACION" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGLAS_HOSPITALES" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGLAS_FEDERACION" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CANDIDATOS_HOSPITALES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CANDIDATOS_FEDERACION" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="REGLAS_HOSPITALES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="REGLAS_FEDERACION" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CANDIDATOS_HOSPITALES'!$A$1:$H$32</definedName>
@@ -2112,7 +2112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2423,7 +2423,11 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2460,7 +2464,11 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2497,7 +2505,11 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2534,7 +2546,11 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="n"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2571,7 +2587,11 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="n"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2608,7 +2628,11 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="n"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2645,7 +2669,11 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="n"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2682,7 +2710,11 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2719,7 +2751,11 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2756,7 +2792,11 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2793,7 +2833,11 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2830,7 +2874,11 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2867,7 +2915,11 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="n"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2904,7 +2956,11 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="n"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2941,7 +2997,11 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="n"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -2978,7 +3038,11 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="n"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -3015,7 +3079,11 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="n"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -3052,7 +3120,11 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="n"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>CASTELLO DE LA PLANA</t>
@@ -3089,7 +3161,11 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3126,7 +3202,11 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="n"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3163,7 +3243,11 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="n"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3200,7 +3284,11 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="n"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3237,7 +3325,11 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="n"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3274,7 +3366,11 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="n"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3311,7 +3407,11 @@
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="n"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3348,7 +3448,11 @@
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="n"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3426,7 +3530,11 @@
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="n"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3463,7 +3571,11 @@
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="n"/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
           <t>VILA-REAL/VILLARREAL</t>
@@ -3496,6 +3608,10 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="n">
         <v>36</v>
@@ -3651,6 +3767,2126 @@
         </is>
       </c>
       <c r="I44" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>BENICASIM S-N</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>BENICASIM S-N</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASÍM, S/N</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASÍM, S/N</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>AVDA BENICASSIM SN</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>AVDA BENICASSIM SN</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>AVGDA. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>AVGDA. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>AV. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>AV. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>AVD. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>AVD. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AV BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>AV BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>AVDA BENICASIM</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>AVDA BENICASIM</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>AVENIDA BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>AVENIDA BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>AVDA DE BENICASIM SN</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>AVDA DE BENICASIM SN</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>DE BENICASIM S/N:HORARIO DE 8.15 A 10.30</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>DE BENICASIM S/N:HORARIO DE 8.15 A 10.30</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>AV .BENICASSIM S/N CASTELLON DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>AV .BENICASSIM S/N CASTELLON DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>53</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM S/N-ALMACENALMACEN</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM S/N-ALMACENALMACEN</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>54</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>55</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>AVD BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>AVD BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>AV BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>AV BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>57</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>AVD BENICASIM, S/N 0</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>AVD BENICASIM, S/N 0</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>58</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>AV.BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>AV.BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>59</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>AVDA. DE BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>AVDA. DE BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>60</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>AV.BENICASSIM,S/N</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>AV.BENICASSIM,S/N</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>AVDA BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>AVDA BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>62</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>AVDA.BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>AVDA.BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>63</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASSIM, S/N - FCIA</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASSIM, S/N - FCIA</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>64</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>AVDA.BENICASIM</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>AVDA.BENICASIM</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>65</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>AV BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>AV BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>AVDA BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>AVDA BENICASIM, S/N</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>AVDA. DE BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>AVDA. DE BENICASSIM S/N</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>AVDA. BENICASSIM, S/N</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>AS DE LA CARRASCA</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>AS DE LA CARRASCA</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>AV. BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>74</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>AV BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>AV BENICASIM S/N</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>75</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ANTA MARIA ROSA MOLAS 25</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>ANTA MARIA ROSA MOLAS 25</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>76</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ANTA MARIA ROSA MOLAS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>ANTA MARIA ROSA MOLAS</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>77</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>FARMACIA C/SANTA MARIA ROSA MOLAS 25 1</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>FARMACIA C/SANTA MARIA ROSA MOLAS 25 1</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>78</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>STA M ROSA MOLAS 25</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>STA M ROSA MOLAS 25</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>REY DON JAIME</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>79</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>RAN VIA TARREGA MONTEBLANCO</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>RAN VIA TARREGA MONTEBLANCO</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>80</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>GRAN VIA TARREGA MONTEBLANCOALMACEN CESQ</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>GRAN VIA TARREGA MONTEBLANCOALMACEN CESQ</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>81</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>AVDA DR CLARA 19</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>AVDA DR CLARA 19</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>82</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>83</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>AVDA. DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>AVDA. DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>84</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>AVENIDA DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>AVENIDA DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>85</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>G.VIA TGA.MONTEBLANCOS,EQ P.JOFRE</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>G.VIA TGA.MONTEBLANCOS,EQ P.JOFRE</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>86</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>PADRE JOFRE ESQUINA CON</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>PADRE JOFRE ESQUINA CON</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>87</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>AVDA DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>AVDA DR. CLARA 19</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>PROVINCIAL</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>88</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>CUADRA COLLET 32 PDA BOVALAR S/N ALMACE</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>CUADRA COLLET 32 PDA BOVALAR S/N ALMACE</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>89</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>CASTELLO DE LA PLANA</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>CR N-340 (CADIZ-BARNA), KM.67 7</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>CR N-340 (CADIZ-BARNA), KM.67 7</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>90</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>VILA-REAL/VILLARREAL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>CTRA DE VILA-REAL A BORRIANA KM 0,5</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>CTRA DE VILA-REAL A BORRIANA KM 0,5</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>91</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>VILA-REAL/VILLARREAL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>CTRA.CV 185 VILLARREAL-BURRIANA KM.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>CTRA.CV 185 VILLARREAL-BURRIANA KM.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>92</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>VILA-REAL/VILLARREAL</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>CR/VILLARREAL A BURRIANA,KM. 0,5 S.FCIA2</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>CR/VILLARREAL A BURRIANA,KM. 0,5 S.FCIA2</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>LA PLANA</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
         <is>
           <t>SI</t>
         </is>

</xml_diff>

<commit_message>
Enriquecer REGLAS_FEDERACION: +20 nuevas variantes de direcciones
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reglas_hospitales.xlsx
+++ b/Reglas_hospitales.xlsx
@@ -3608,10 +3608,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" t="n">
         <v>36</v>
@@ -5904,7 +5900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6639,6 +6635,18 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="n">
         <v>18</v>
@@ -6794,6 +6802,726 @@
         </is>
       </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>22</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CALLE SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>CALLE SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>23</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>C/ STA. QUITERIA, 342 P.I. MIJARES, PARC</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>C/ STA. QUITERIA, 342 P.I. MIJARES, PARC</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>24</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>C/ STA. QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>C/ STA. QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>25</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CL SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>CL SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>26</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CL/ STA. QUITERIA, 342, P. I. MIJARES</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>CL/ STA. QUITERIA, 342, P. I. MIJARES</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>27</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>28</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA, 342</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>29</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA, 342-C/ L'ALCORA,</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>C/ SANTA QUITERIA, 342-C/ L'ALCORA,</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>30</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>C/SANTA QUITERIA. 342</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>C/SANTA QUITERIA. 342</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>31</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>C/SANTA QUITERÍA, 342</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>C/SANTA QUITERÍA, 342</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>32</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CL STA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CL STA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>33</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CL. SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>CL. SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>34</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>SANTA QUITERÍA, 342</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SANTA QUITERÍA, 342</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>35</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>STA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>STA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>36</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SANTA QUITERIA 342</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>37</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P MIJARES-PARCELA 16</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>P MIJARES-PARCELA 16</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>38</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>PG IND. MIJARES PARC. 17- 19</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PG IND. MIJARES PARC. 17- 19</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>39</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CL ALCORA, 282</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>CL ALCORA, 282</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>40</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CL,ALCORA 282</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CL,ALCORA 282</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>41</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>FEDERACION</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ALMASSORA/ALMAZORA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CARRER DE L ALCORA, 282 -</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FEDERAC</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>CARRER DE L ALCORA, 282 -</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
         <is>
           <t>SI</t>
         </is>

</xml_diff>